<commit_message>
Update vaccine data, outputs, and figure label
Updated Data/VaccineSchedule.xlsx and regenerated output files (Output/Figure 1.xlsx, Output/Figure 3.pdf, Output/Figure 3.xlsx). Cleaned Output/Table S1.csv by removing the leading index/empty column so the header now starts with ISO3. Adjusted Script/figure3.R to change the x-axis label from 'Recommended time for maternal vaccination (weeks)' to 'Gestational week of vaccination'.
</commit_message>
<xml_diff>
--- a/Data/VaccineSchedule.xlsx
+++ b/Data/VaccineSchedule.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://6kmwxn-my.sharepoint.com/personal/kanggle_globalinfectiousdisease_com/Documents/XMU/likangguo/2025/28 百日咳数据对比/Project/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="710" documentId="8_{6B2C8828-AD43-45C3-B957-8962AC28D08B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ED4AAA81-4060-4DC4-A9DC-31B972608786}"/>
+  <xr:revisionPtr revIDLastSave="711" documentId="8_{6B2C8828-AD43-45C3-B957-8962AC28D08B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AC357534-91CA-4978-9A49-3F288B01583F}"/>
   <bookViews>
-    <workbookView xWindow="-797" yWindow="2254" windowWidth="19423" windowHeight="12420" xr2:uid="{04EA11F9-B7BC-471A-98F9-2CFDCD6CFD79}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="29020" windowHeight="15820" xr2:uid="{04EA11F9-B7BC-471A-98F9-2CFDCD6CFD79}"/>
   </bookViews>
   <sheets>
     <sheet name="VaccineSchedule" sheetId="1" r:id="rId1"/>
@@ -1505,6 +1505,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="176" formatCode="0.00_ "/>
+  </numFmts>
   <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -2106,7 +2109,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -2118,6 +2121,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="43">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -2167,7 +2173,13 @@
     <cellStyle name="着色 6" xfId="38" builtinId="49" customBuiltin="1"/>
     <cellStyle name="注释" xfId="15" builtinId="10" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="3">
+    <dxf>
+      <numFmt numFmtId="176" formatCode="0.00_ "/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="176" formatCode="0.00_ "/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
@@ -2195,11 +2207,11 @@
     <tableColumn id="12" xr3:uid="{91A80A45-CDFC-4097-B30C-0318DEA5773D}" name="VaccinePregnantSource"/>
     <tableColumn id="4" xr3:uid="{28571980-2668-4B5D-B850-849FF73305BE}" name="VaccineAdult"/>
     <tableColumn id="5" xr3:uid="{40B31AF5-542D-4D82-B761-6464158DAF1E}" name="VaccineRisk"/>
-    <tableColumn id="6" xr3:uid="{6518DF24-B97F-4720-BA8E-2B5AC278AA41}" name="TimeLastShot"/>
-    <tableColumn id="7" xr3:uid="{0B12E78F-93A1-4BC4-8CC5-8583B74E4789}" name="TimeFirstShot"/>
+    <tableColumn id="6" xr3:uid="{6518DF24-B97F-4720-BA8E-2B5AC278AA41}" name="TimeLastShot" dataDxfId="1"/>
+    <tableColumn id="7" xr3:uid="{0B12E78F-93A1-4BC4-8CC5-8583B74E4789}" name="TimeFirstShot" dataDxfId="0"/>
     <tableColumn id="8" xr3:uid="{024744F4-9A3D-45D3-AF1D-8742303F2F62}" name="VaccineDose1"/>
     <tableColumn id="10" xr3:uid="{4E47E6AC-697F-416A-88DC-F42D0EB077AC}" name="VaccineDose2"/>
-    <tableColumn id="11" xr3:uid="{CDC544EF-5E48-406E-875C-544F76F4E642}" name="VaccineDose" dataDxfId="0">
+    <tableColumn id="11" xr3:uid="{CDC544EF-5E48-406E-875C-544F76F4E642}" name="VaccineDose" dataDxfId="2">
       <calculatedColumnFormula>IF(表1[[#This Row],[VaccineDose1]]=表1[[#This Row],[VaccineDose2]],表1[[#This Row],[VaccineDose1]],99)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2531,8 +2543,8 @@
     <col min="3" max="5" width="15.58203125" customWidth="1"/>
     <col min="6" max="6" width="12.83203125" customWidth="1"/>
     <col min="7" max="7" width="11.58203125" customWidth="1"/>
-    <col min="8" max="8" width="13.08203125" customWidth="1"/>
-    <col min="9" max="9" width="17.33203125" customWidth="1"/>
+    <col min="8" max="8" width="13.08203125" style="5" customWidth="1"/>
+    <col min="9" max="9" width="17.33203125" style="5" customWidth="1"/>
     <col min="10" max="10" width="15.08203125" customWidth="1"/>
     <col min="11" max="12" width="9.58203125" customWidth="1"/>
   </cols>
@@ -2559,10 +2571,10 @@
       <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="5" t="s">
         <v>8</v>
       </c>
       <c r="J1" t="s">
@@ -2591,10 +2603,10 @@
       <c r="G2">
         <v>1</v>
       </c>
-      <c r="H2">
+      <c r="H2" s="5">
         <v>120</v>
       </c>
-      <c r="I2">
+      <c r="I2" s="5">
         <v>2</v>
       </c>
       <c r="J2">
@@ -2624,10 +2636,10 @@
       <c r="G3">
         <v>0</v>
       </c>
-      <c r="H3">
+      <c r="H3" s="5">
         <v>3.2183908045976999</v>
       </c>
-      <c r="I3">
+      <c r="I3" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J3">
@@ -2657,10 +2669,10 @@
       <c r="G4">
         <v>0</v>
       </c>
-      <c r="H4">
-        <v>6</v>
-      </c>
-      <c r="I4">
+      <c r="H4" s="5">
+        <v>6</v>
+      </c>
+      <c r="I4" s="5">
         <v>2</v>
       </c>
       <c r="J4">
@@ -2690,10 +2702,10 @@
       <c r="G5">
         <v>1</v>
       </c>
-      <c r="H5">
+      <c r="H5" s="5">
         <v>60</v>
       </c>
-      <c r="I5">
+      <c r="I5" s="5">
         <v>2</v>
       </c>
       <c r="J5">
@@ -2723,10 +2735,10 @@
       <c r="G6">
         <v>0</v>
       </c>
-      <c r="H6">
+      <c r="H6" s="5">
         <v>24</v>
       </c>
-      <c r="I6">
+      <c r="I6" s="5">
         <v>2</v>
       </c>
       <c r="J6">
@@ -2762,10 +2774,10 @@
       <c r="G7">
         <v>0</v>
       </c>
-      <c r="H7">
+      <c r="H7" s="5">
         <v>180</v>
       </c>
-      <c r="I7">
+      <c r="I7" s="5">
         <v>2</v>
       </c>
       <c r="J7">
@@ -2795,10 +2807,10 @@
       <c r="G8">
         <v>1</v>
       </c>
-      <c r="H8">
+      <c r="H8" s="5">
         <v>192</v>
       </c>
-      <c r="I8">
+      <c r="I8" s="5">
         <v>2</v>
       </c>
       <c r="J8">
@@ -2834,10 +2846,10 @@
       <c r="G9">
         <v>1</v>
       </c>
-      <c r="H9">
+      <c r="H9" s="5">
         <v>132</v>
       </c>
-      <c r="I9">
+      <c r="I9" s="5">
         <v>2</v>
       </c>
       <c r="J9">
@@ -2867,10 +2879,10 @@
       <c r="G10">
         <v>0</v>
       </c>
-      <c r="H10">
+      <c r="H10" s="5">
         <v>192</v>
       </c>
-      <c r="I10">
+      <c r="I10" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J10">
@@ -2900,10 +2912,10 @@
       <c r="G11">
         <v>0</v>
       </c>
-      <c r="H11">
+      <c r="H11" s="5">
         <v>18</v>
       </c>
-      <c r="I11">
+      <c r="I11" s="5">
         <v>2</v>
       </c>
       <c r="J11">
@@ -2939,10 +2951,10 @@
       <c r="G12">
         <v>0</v>
       </c>
-      <c r="H12">
+      <c r="H12" s="5">
         <v>156</v>
       </c>
-      <c r="I12">
+      <c r="I12" s="5">
         <v>2</v>
       </c>
       <c r="J12">
@@ -2978,10 +2990,10 @@
       <c r="G13">
         <v>0</v>
       </c>
-      <c r="H13">
+      <c r="H13" s="5">
         <v>96</v>
       </c>
-      <c r="I13">
+      <c r="I13" s="5">
         <v>2</v>
       </c>
       <c r="J13">
@@ -3011,10 +3023,10 @@
       <c r="G14">
         <v>0</v>
       </c>
-      <c r="H14">
+      <c r="H14" s="5">
         <v>18</v>
       </c>
-      <c r="I14">
+      <c r="I14" s="5">
         <v>2</v>
       </c>
       <c r="J14">
@@ -3044,10 +3056,10 @@
       <c r="G15">
         <v>0</v>
       </c>
-      <c r="H15">
+      <c r="H15" s="5">
         <v>18</v>
       </c>
-      <c r="I15">
+      <c r="I15" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J15">
@@ -3083,10 +3095,10 @@
       <c r="G16">
         <v>0</v>
       </c>
-      <c r="H16">
+      <c r="H16" s="5">
         <v>192</v>
       </c>
-      <c r="I16">
+      <c r="I16" s="5">
         <v>1.83908045977012</v>
       </c>
       <c r="J16">
@@ -3116,10 +3128,10 @@
       <c r="G17">
         <v>0</v>
       </c>
-      <c r="H17">
+      <c r="H17" s="5">
         <v>3.2183908045976999</v>
       </c>
-      <c r="I17">
+      <c r="I17" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J17">
@@ -3149,10 +3161,10 @@
       <c r="G18">
         <v>0</v>
       </c>
-      <c r="H18">
+      <c r="H18" s="5">
         <v>3.6781609195402298</v>
       </c>
-      <c r="I18">
+      <c r="I18" s="5">
         <v>1.83908045977012</v>
       </c>
       <c r="J18">
@@ -3182,10 +3194,10 @@
       <c r="G19">
         <v>0</v>
       </c>
-      <c r="H19">
+      <c r="H19" s="5">
         <v>3.2183908045976999</v>
       </c>
-      <c r="I19">
+      <c r="I19" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J19">
@@ -3215,10 +3227,10 @@
       <c r="G20">
         <v>0</v>
       </c>
-      <c r="H20">
+      <c r="H20" s="5">
         <v>144</v>
       </c>
-      <c r="I20">
+      <c r="I20" s="5">
         <v>2</v>
       </c>
       <c r="J20">
@@ -3248,10 +3260,10 @@
       <c r="G21">
         <v>1</v>
       </c>
-      <c r="H21">
+      <c r="H21" s="5">
         <v>156</v>
       </c>
-      <c r="I21">
+      <c r="I21" s="5">
         <v>2</v>
       </c>
       <c r="J21">
@@ -3287,10 +3299,10 @@
       <c r="G22">
         <v>0</v>
       </c>
-      <c r="H22">
+      <c r="H22" s="5">
         <v>144</v>
       </c>
-      <c r="I22">
+      <c r="I22" s="5">
         <v>2</v>
       </c>
       <c r="J22">
@@ -3320,10 +3332,10 @@
       <c r="G23">
         <v>0</v>
       </c>
-      <c r="H23">
+      <c r="H23" s="5">
         <v>84</v>
       </c>
-      <c r="I23">
+      <c r="I23" s="5">
         <v>2</v>
       </c>
       <c r="J23">
@@ -3353,10 +3365,10 @@
       <c r="G24">
         <v>1</v>
       </c>
-      <c r="H24">
+      <c r="H24" s="5">
         <v>18</v>
       </c>
-      <c r="I24">
+      <c r="I24" s="5">
         <v>2</v>
       </c>
       <c r="J24">
@@ -3386,10 +3398,10 @@
       <c r="G25">
         <v>0</v>
       </c>
-      <c r="H25">
+      <c r="H25" s="5">
         <v>48</v>
       </c>
-      <c r="I25">
+      <c r="I25" s="5">
         <v>2</v>
       </c>
       <c r="J25">
@@ -3425,10 +3437,10 @@
       <c r="G26">
         <v>0</v>
       </c>
-      <c r="H26">
+      <c r="H26" s="5">
         <v>216</v>
       </c>
-      <c r="I26">
+      <c r="I26" s="5">
         <v>2</v>
       </c>
       <c r="J26">
@@ -3458,10 +3470,10 @@
       <c r="G27">
         <v>0</v>
       </c>
-      <c r="H27">
+      <c r="H27" s="5">
         <v>48</v>
       </c>
-      <c r="I27">
+      <c r="I27" s="5">
         <v>2</v>
       </c>
       <c r="J27">
@@ -3497,10 +3509,10 @@
       <c r="G28">
         <v>1</v>
       </c>
-      <c r="H28">
+      <c r="H28" s="5">
         <v>48</v>
       </c>
-      <c r="I28">
+      <c r="I28" s="5">
         <v>2</v>
       </c>
       <c r="J28">
@@ -3530,10 +3542,10 @@
       <c r="G29">
         <v>1</v>
       </c>
-      <c r="H29">
+      <c r="H29" s="5">
         <v>54</v>
       </c>
-      <c r="I29">
+      <c r="I29" s="5">
         <v>2</v>
       </c>
       <c r="J29">
@@ -3563,10 +3575,10 @@
       <c r="G30">
         <v>0</v>
       </c>
-      <c r="H30">
+      <c r="H30" s="5">
         <v>60</v>
       </c>
-      <c r="I30">
+      <c r="I30" s="5">
         <v>2</v>
       </c>
       <c r="J30">
@@ -3596,10 +3608,10 @@
       <c r="G31">
         <v>0</v>
       </c>
-      <c r="H31">
+      <c r="H31" s="5">
         <v>24</v>
       </c>
-      <c r="I31">
+      <c r="I31" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J31">
@@ -3629,10 +3641,10 @@
       <c r="G32">
         <v>0</v>
       </c>
-      <c r="H32">
-        <v>4</v>
-      </c>
-      <c r="I32">
+      <c r="H32" s="5">
+        <v>4</v>
+      </c>
+      <c r="I32" s="5">
         <v>2</v>
       </c>
       <c r="J32">
@@ -3662,10 +3674,10 @@
       <c r="G33">
         <v>0</v>
       </c>
-      <c r="H33">
+      <c r="H33" s="5">
         <v>3.2183908045976999</v>
       </c>
-      <c r="I33">
+      <c r="I33" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J33">
@@ -3701,10 +3713,10 @@
       <c r="G34">
         <v>0</v>
       </c>
-      <c r="H34">
+      <c r="H34" s="5">
         <v>192</v>
       </c>
-      <c r="I34">
+      <c r="I34" s="5">
         <v>2</v>
       </c>
       <c r="J34">
@@ -3740,10 +3752,10 @@
       <c r="G35">
         <v>0</v>
       </c>
-      <c r="H35">
+      <c r="H35" s="5">
         <v>180</v>
       </c>
-      <c r="I35">
+      <c r="I35" s="5">
         <v>2</v>
       </c>
       <c r="J35">
@@ -3779,10 +3791,10 @@
       <c r="G36">
         <v>0</v>
       </c>
-      <c r="H36">
+      <c r="H36" s="5">
         <v>156</v>
       </c>
-      <c r="I36">
+      <c r="I36" s="5">
         <v>2</v>
       </c>
       <c r="J36">
@@ -3812,10 +3824,10 @@
       <c r="G37">
         <v>0</v>
       </c>
-      <c r="H37">
+      <c r="H37" s="5">
         <v>18</v>
       </c>
-      <c r="I37">
+      <c r="I37" s="5">
         <v>3</v>
       </c>
       <c r="J37">
@@ -3845,10 +3857,10 @@
       <c r="G38">
         <v>0</v>
       </c>
-      <c r="H38">
+      <c r="H38" s="5">
         <v>3.2183908045976999</v>
       </c>
-      <c r="I38">
+      <c r="I38" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J38">
@@ -3878,10 +3890,10 @@
       <c r="G39">
         <v>0</v>
       </c>
-      <c r="H39">
+      <c r="H39" s="5">
         <v>3.2183908045976999</v>
       </c>
-      <c r="I39">
+      <c r="I39" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J39">
@@ -3911,10 +3923,10 @@
       <c r="G40">
         <v>0</v>
       </c>
-      <c r="H40">
+      <c r="H40" s="5">
         <v>3.2183908045976999</v>
       </c>
-      <c r="I40">
+      <c r="I40" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J40">
@@ -3944,10 +3956,10 @@
       <c r="G41">
         <v>0</v>
       </c>
-      <c r="H41">
+      <c r="H41" s="5">
         <v>3.6781609195402298</v>
       </c>
-      <c r="I41">
+      <c r="I41" s="5">
         <v>1.83908045977012</v>
       </c>
       <c r="J41">
@@ -3977,10 +3989,10 @@
       <c r="G42">
         <v>0</v>
       </c>
-      <c r="H42">
+      <c r="H42" s="5">
         <v>48</v>
       </c>
-      <c r="I42">
+      <c r="I42" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J42">
@@ -4016,10 +4028,10 @@
       <c r="G43">
         <v>1</v>
       </c>
-      <c r="H43">
+      <c r="H43" s="5">
         <v>18</v>
       </c>
-      <c r="I43">
+      <c r="I43" s="5">
         <v>2</v>
       </c>
       <c r="J43">
@@ -4049,10 +4061,10 @@
       <c r="G44">
         <v>0</v>
       </c>
-      <c r="H44">
+      <c r="H44" s="5">
         <v>3.2183908045976999</v>
       </c>
-      <c r="I44">
+      <c r="I44" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J44">
@@ -4082,10 +4094,10 @@
       <c r="G45">
         <v>0</v>
       </c>
-      <c r="H45">
+      <c r="H45" s="5">
         <v>18</v>
       </c>
-      <c r="I45">
+      <c r="I45" s="5">
         <v>2</v>
       </c>
       <c r="J45">
@@ -4121,10 +4133,10 @@
       <c r="G46">
         <v>1</v>
       </c>
-      <c r="H46">
+      <c r="H46" s="5">
         <v>48</v>
       </c>
-      <c r="I46">
+      <c r="I46" s="5">
         <v>2</v>
       </c>
       <c r="J46">
@@ -4154,10 +4166,10 @@
       <c r="G47">
         <v>1</v>
       </c>
-      <c r="H47">
+      <c r="H47" s="5">
         <v>18</v>
       </c>
-      <c r="I47">
+      <c r="I47" s="5">
         <v>2</v>
       </c>
       <c r="J47">
@@ -4187,10 +4199,10 @@
       <c r="G48">
         <v>0</v>
       </c>
-      <c r="H48">
+      <c r="H48" s="5">
         <v>15</v>
       </c>
-      <c r="I48">
+      <c r="I48" s="5">
         <v>2</v>
       </c>
       <c r="J48">
@@ -4226,10 +4238,10 @@
       <c r="G49">
         <v>0</v>
       </c>
-      <c r="H49">
+      <c r="H49" s="5">
         <v>192</v>
       </c>
-      <c r="I49">
+      <c r="I49" s="5">
         <v>2</v>
       </c>
       <c r="J49">
@@ -4265,10 +4277,10 @@
       <c r="G50">
         <v>0</v>
       </c>
-      <c r="H50">
+      <c r="H50" s="5">
         <v>144</v>
       </c>
-      <c r="I50">
+      <c r="I50" s="5">
         <v>2</v>
       </c>
       <c r="J50">
@@ -4298,10 +4310,10 @@
       <c r="G51">
         <v>0</v>
       </c>
-      <c r="H51">
+      <c r="H51" s="5">
         <v>120</v>
       </c>
-      <c r="I51">
+      <c r="I51" s="5">
         <v>3</v>
       </c>
       <c r="J51">
@@ -4337,10 +4349,10 @@
       <c r="G52">
         <v>1</v>
       </c>
-      <c r="H52">
+      <c r="H52" s="5">
         <v>192</v>
       </c>
-      <c r="I52">
+      <c r="I52" s="5">
         <v>2</v>
       </c>
       <c r="J52">
@@ -4370,10 +4382,10 @@
       <c r="G53">
         <v>0</v>
       </c>
-      <c r="H53">
+      <c r="H53" s="5">
         <v>15</v>
       </c>
-      <c r="I53">
+      <c r="I53" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J53">
@@ -4403,10 +4415,10 @@
       <c r="G54">
         <v>0</v>
       </c>
-      <c r="H54">
+      <c r="H54" s="5">
         <v>36</v>
       </c>
-      <c r="I54">
+      <c r="I54" s="5">
         <v>2</v>
       </c>
       <c r="J54">
@@ -4436,10 +4448,10 @@
       <c r="G55">
         <v>0</v>
       </c>
-      <c r="H55">
+      <c r="H55" s="5">
         <v>60</v>
       </c>
-      <c r="I55">
+      <c r="I55" s="5">
         <v>3</v>
       </c>
       <c r="J55">
@@ -4475,10 +4487,10 @@
       <c r="G56">
         <v>1</v>
       </c>
-      <c r="H56">
+      <c r="H56" s="5">
         <v>48</v>
       </c>
-      <c r="I56">
+      <c r="I56" s="5">
         <v>2</v>
       </c>
       <c r="J56">
@@ -4508,10 +4520,10 @@
       <c r="G57">
         <v>0</v>
       </c>
-      <c r="H57">
+      <c r="H57" s="5">
         <v>72</v>
       </c>
-      <c r="I57">
+      <c r="I57" s="5">
         <v>2</v>
       </c>
       <c r="J57">
@@ -4541,10 +4553,10 @@
       <c r="G58">
         <v>0</v>
       </c>
-      <c r="H58">
+      <c r="H58" s="5">
         <v>60</v>
       </c>
-      <c r="I58">
+      <c r="I58" s="5">
         <v>2</v>
       </c>
       <c r="J58">
@@ -4574,10 +4586,10 @@
       <c r="G59">
         <v>0</v>
       </c>
-      <c r="H59">
+      <c r="H59" s="5">
         <v>18</v>
       </c>
-      <c r="I59">
+      <c r="I59" s="5">
         <v>2</v>
       </c>
       <c r="J59">
@@ -4607,10 +4619,10 @@
       <c r="G60">
         <v>0</v>
       </c>
-      <c r="H60">
+      <c r="H60" s="5">
         <v>3.2183908045976999</v>
       </c>
-      <c r="I60">
+      <c r="I60" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J60">
@@ -4646,10 +4658,10 @@
       <c r="G61">
         <v>1</v>
       </c>
-      <c r="H61">
+      <c r="H61" s="5">
         <v>72</v>
       </c>
-      <c r="I61">
+      <c r="I61" s="5">
         <v>2</v>
       </c>
       <c r="J61">
@@ -4679,10 +4691,10 @@
       <c r="G62">
         <v>0</v>
       </c>
-      <c r="H62">
+      <c r="H62" s="5">
         <v>192</v>
       </c>
-      <c r="I62">
+      <c r="I62" s="5">
         <v>3</v>
       </c>
       <c r="J62">
@@ -4712,10 +4724,10 @@
       <c r="G63">
         <v>0</v>
       </c>
-      <c r="H63">
+      <c r="H63" s="5">
         <v>3.2183908045976999</v>
       </c>
-      <c r="I63">
+      <c r="I63" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J63">
@@ -4745,10 +4757,10 @@
       <c r="G64">
         <v>0</v>
       </c>
-      <c r="H64">
+      <c r="H64" s="5">
         <v>180</v>
       </c>
-      <c r="I64">
+      <c r="I64" s="5">
         <v>3</v>
       </c>
       <c r="J64">
@@ -4778,10 +4790,10 @@
       <c r="G65">
         <v>0</v>
       </c>
-      <c r="H65">
+      <c r="H65" s="5">
         <v>3.2183908045976999</v>
       </c>
-      <c r="I65">
+      <c r="I65" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J65">
@@ -4817,10 +4829,10 @@
       <c r="G66">
         <v>0</v>
       </c>
-      <c r="H66">
+      <c r="H66" s="5">
         <v>156</v>
       </c>
-      <c r="I66">
+      <c r="I66" s="5">
         <v>2</v>
       </c>
       <c r="J66">
@@ -4850,10 +4862,10 @@
       <c r="G67">
         <v>0</v>
       </c>
-      <c r="H67">
+      <c r="H67" s="5">
         <v>144</v>
       </c>
-      <c r="I67">
+      <c r="I67" s="5">
         <v>2</v>
       </c>
       <c r="J67">
@@ -4883,10 +4895,10 @@
       <c r="G68">
         <v>0</v>
       </c>
-      <c r="H68">
+      <c r="H68" s="5">
         <v>3.2183908045976999</v>
       </c>
-      <c r="I68">
+      <c r="I68" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J68">
@@ -4922,10 +4934,10 @@
       <c r="G69">
         <v>0</v>
       </c>
-      <c r="H69">
+      <c r="H69" s="5">
         <v>40</v>
       </c>
-      <c r="I69">
+      <c r="I69" s="5">
         <v>1.83908045977012</v>
       </c>
       <c r="J69">
@@ -4955,10 +4967,10 @@
       <c r="G70">
         <v>0</v>
       </c>
-      <c r="H70">
+      <c r="H70" s="5">
         <v>60</v>
       </c>
-      <c r="I70">
+      <c r="I70" s="5">
         <v>2</v>
       </c>
       <c r="J70">
@@ -4988,10 +5000,10 @@
       <c r="G71">
         <v>0</v>
       </c>
-      <c r="H71">
+      <c r="H71" s="5">
         <v>3.2183908045976999</v>
       </c>
-      <c r="I71">
+      <c r="I71" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J71">
@@ -5021,10 +5033,10 @@
       <c r="G72">
         <v>0</v>
       </c>
-      <c r="H72">
+      <c r="H72" s="5">
         <v>3.2183908045976999</v>
       </c>
-      <c r="I72">
+      <c r="I72" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J72">
@@ -5054,10 +5066,10 @@
       <c r="G73">
         <v>0</v>
       </c>
-      <c r="H73">
+      <c r="H73" s="5">
         <v>18</v>
       </c>
-      <c r="I73">
+      <c r="I73" s="5">
         <v>2</v>
       </c>
       <c r="J73">
@@ -5087,10 +5099,10 @@
       <c r="G74">
         <v>0</v>
       </c>
-      <c r="H74">
+      <c r="H74" s="5">
         <v>3.2183908045976999</v>
       </c>
-      <c r="I74">
+      <c r="I74" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J74">
@@ -5120,10 +5132,10 @@
       <c r="G75">
         <v>0</v>
       </c>
-      <c r="H75">
+      <c r="H75" s="5">
         <v>18</v>
       </c>
-      <c r="I75">
+      <c r="I75" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J75">
@@ -5153,10 +5165,10 @@
       <c r="G76">
         <v>0</v>
       </c>
-      <c r="H76">
+      <c r="H76" s="5">
         <v>144</v>
       </c>
-      <c r="I76">
+      <c r="I76" s="5">
         <v>2</v>
       </c>
       <c r="J76">
@@ -5186,10 +5198,10 @@
       <c r="G77">
         <v>0</v>
       </c>
-      <c r="H77">
+      <c r="H77" s="5">
         <v>18</v>
       </c>
-      <c r="I77">
+      <c r="I77" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J77">
@@ -5225,10 +5237,10 @@
       <c r="G78">
         <v>1</v>
       </c>
-      <c r="H78">
+      <c r="H78" s="5">
         <v>48</v>
       </c>
-      <c r="I78">
+      <c r="I78" s="5">
         <v>2</v>
       </c>
       <c r="J78">
@@ -5264,10 +5276,10 @@
       <c r="G79">
         <v>0</v>
       </c>
-      <c r="H79">
+      <c r="H79" s="5">
         <v>132</v>
       </c>
-      <c r="I79">
+      <c r="I79" s="5">
         <v>2</v>
       </c>
       <c r="J79">
@@ -5297,10 +5309,10 @@
       <c r="G80">
         <v>0</v>
       </c>
-      <c r="H80">
-        <v>6</v>
-      </c>
-      <c r="I80">
+      <c r="H80" s="5">
+        <v>6</v>
+      </c>
+      <c r="I80" s="5">
         <v>2</v>
       </c>
       <c r="J80">
@@ -5336,10 +5348,10 @@
       <c r="G81">
         <v>0</v>
       </c>
-      <c r="H81">
+      <c r="H81" s="5">
         <v>132</v>
       </c>
-      <c r="I81">
+      <c r="I81" s="5">
         <v>2</v>
       </c>
       <c r="J81">
@@ -5375,10 +5387,10 @@
       <c r="G82">
         <v>1</v>
       </c>
-      <c r="H82">
+      <c r="H82" s="5">
         <v>48</v>
       </c>
-      <c r="I82">
+      <c r="I82" s="5">
         <v>2</v>
       </c>
       <c r="J82">
@@ -5408,10 +5420,10 @@
       <c r="G83">
         <v>0</v>
       </c>
-      <c r="H83">
+      <c r="H83" s="5">
         <v>72</v>
       </c>
-      <c r="I83">
+      <c r="I83" s="5">
         <v>2</v>
       </c>
       <c r="J83">
@@ -5441,10 +5453,10 @@
       <c r="G84">
         <v>0</v>
       </c>
-      <c r="H84">
+      <c r="H84" s="5">
         <v>15</v>
       </c>
-      <c r="I84">
+      <c r="I84" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J84">
@@ -5480,10 +5492,10 @@
       <c r="G85">
         <v>0</v>
       </c>
-      <c r="H85">
+      <c r="H85" s="5">
         <v>132</v>
       </c>
-      <c r="I85">
+      <c r="I85" s="5">
         <v>2</v>
       </c>
       <c r="J85">
@@ -5513,10 +5525,10 @@
       <c r="G86">
         <v>0</v>
       </c>
-      <c r="H86">
+      <c r="H86" s="5">
         <v>18</v>
       </c>
-      <c r="I86">
+      <c r="I86" s="5">
         <v>2</v>
       </c>
       <c r="J86">
@@ -5552,10 +5564,10 @@
       <c r="G87">
         <v>0</v>
       </c>
-      <c r="H87">
+      <c r="H87" s="5">
         <v>72</v>
       </c>
-      <c r="I87">
+      <c r="I87" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J87">
@@ -5591,10 +5603,10 @@
       <c r="G88">
         <v>1</v>
       </c>
-      <c r="H88">
+      <c r="H88" s="5">
         <v>156</v>
       </c>
-      <c r="I88">
+      <c r="I88" s="5">
         <v>2</v>
       </c>
       <c r="J88">
@@ -5624,10 +5636,10 @@
       <c r="G89">
         <v>0</v>
       </c>
-      <c r="H89">
+      <c r="H89" s="5">
         <v>72</v>
       </c>
-      <c r="I89">
+      <c r="I89" s="5">
         <v>2</v>
       </c>
       <c r="J89">
@@ -5657,10 +5669,10 @@
       <c r="G90">
         <v>0</v>
       </c>
-      <c r="H90">
+      <c r="H90" s="5">
         <v>72</v>
       </c>
-      <c r="I90">
+      <c r="I90" s="5">
         <v>2</v>
       </c>
       <c r="J90">
@@ -5696,10 +5708,10 @@
       <c r="G91">
         <v>0</v>
       </c>
-      <c r="H91">
+      <c r="H91" s="5">
         <v>168</v>
       </c>
-      <c r="I91">
+      <c r="I91" s="5">
         <v>3</v>
       </c>
       <c r="J91">
@@ -5735,10 +5747,10 @@
       <c r="G92">
         <v>1</v>
       </c>
-      <c r="H92">
+      <c r="H92" s="5">
         <v>156</v>
       </c>
-      <c r="I92">
+      <c r="I92" s="5">
         <v>2</v>
       </c>
       <c r="J92">
@@ -5774,10 +5786,10 @@
       <c r="G93">
         <v>0</v>
       </c>
-      <c r="H93">
+      <c r="H93" s="5">
         <v>216</v>
       </c>
-      <c r="I93">
+      <c r="I93" s="5">
         <v>3</v>
       </c>
       <c r="J93">
@@ -5807,10 +5819,10 @@
       <c r="G94">
         <v>0</v>
       </c>
-      <c r="H94">
+      <c r="H94" s="5">
         <v>72</v>
       </c>
-      <c r="I94">
+      <c r="I94" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J94">
@@ -5840,10 +5852,10 @@
       <c r="G95">
         <v>0</v>
       </c>
-      <c r="H95">
+      <c r="H95" s="5">
         <v>18</v>
       </c>
-      <c r="I95">
+      <c r="I95" s="5">
         <v>3</v>
       </c>
       <c r="J95">
@@ -5873,10 +5885,10 @@
       <c r="G96">
         <v>0</v>
       </c>
-      <c r="H96">
+      <c r="H96" s="5">
         <v>18</v>
       </c>
-      <c r="I96">
+      <c r="I96" s="5">
         <v>3</v>
       </c>
       <c r="J96">
@@ -5906,10 +5918,10 @@
       <c r="G97">
         <v>0</v>
       </c>
-      <c r="H97">
+      <c r="H97" s="5">
         <v>72</v>
       </c>
-      <c r="I97">
+      <c r="I97" s="5">
         <v>2</v>
       </c>
       <c r="J97">
@@ -5939,10 +5951,10 @@
       <c r="G98">
         <v>0</v>
       </c>
-      <c r="H98">
+      <c r="H98" s="5">
         <v>3.2183908045976999</v>
       </c>
-      <c r="I98">
+      <c r="I98" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J98">
@@ -5972,10 +5984,10 @@
       <c r="G99">
         <v>0</v>
       </c>
-      <c r="H99">
+      <c r="H99" s="5">
         <v>24</v>
       </c>
-      <c r="I99">
+      <c r="I99" s="5">
         <v>2</v>
       </c>
       <c r="J99">
@@ -6005,10 +6017,10 @@
       <c r="G100">
         <v>0</v>
       </c>
-      <c r="H100">
+      <c r="H100" s="5">
         <v>3.2183908045976999</v>
       </c>
-      <c r="I100">
+      <c r="I100" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J100">
@@ -6038,10 +6050,10 @@
       <c r="G101">
         <v>0</v>
       </c>
-      <c r="H101">
+      <c r="H101" s="5">
         <v>72</v>
       </c>
-      <c r="I101">
+      <c r="I101" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J101">
@@ -6071,10 +6083,10 @@
       <c r="G102">
         <v>0</v>
       </c>
-      <c r="H102">
+      <c r="H102" s="5">
         <v>60</v>
       </c>
-      <c r="I102">
+      <c r="I102" s="5">
         <v>2</v>
       </c>
       <c r="J102">
@@ -6104,10 +6116,10 @@
       <c r="G103">
         <v>0</v>
       </c>
-      <c r="H103">
+      <c r="H103" s="5">
         <v>144</v>
       </c>
-      <c r="I103">
+      <c r="I103" s="5">
         <v>2</v>
       </c>
       <c r="J103">
@@ -6137,10 +6149,10 @@
       <c r="G104">
         <v>0</v>
       </c>
-      <c r="H104">
+      <c r="H104" s="5">
         <v>43.2</v>
       </c>
-      <c r="I104">
+      <c r="I104" s="5">
         <v>2</v>
       </c>
       <c r="J104">
@@ -6170,10 +6182,10 @@
       <c r="G105">
         <v>0</v>
       </c>
-      <c r="H105">
+      <c r="H105" s="5">
         <v>3.2183908045976999</v>
       </c>
-      <c r="I105">
+      <c r="I105" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J105">
@@ -6203,10 +6215,10 @@
       <c r="G106">
         <v>0</v>
       </c>
-      <c r="H106">
+      <c r="H106" s="5">
         <v>60</v>
       </c>
-      <c r="I106">
+      <c r="I106" s="5">
         <v>2</v>
       </c>
       <c r="J106">
@@ -6236,10 +6248,10 @@
       <c r="G107">
         <v>0</v>
       </c>
-      <c r="H107">
+      <c r="H107" s="5">
         <v>3.2183908045976999</v>
       </c>
-      <c r="I107">
+      <c r="I107" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J107">
@@ -6269,10 +6281,10 @@
       <c r="G108">
         <v>0</v>
       </c>
-      <c r="H108">
+      <c r="H108" s="5">
         <v>180</v>
       </c>
-      <c r="I108">
+      <c r="I108" s="5">
         <v>2</v>
       </c>
       <c r="J108">
@@ -6302,10 +6314,10 @@
       <c r="G109">
         <v>0</v>
       </c>
-      <c r="H109">
+      <c r="H109" s="5">
         <v>60</v>
       </c>
-      <c r="I109">
+      <c r="I109" s="5">
         <v>2</v>
       </c>
       <c r="J109">
@@ -6335,10 +6347,10 @@
       <c r="G110">
         <v>0</v>
       </c>
-      <c r="H110">
+      <c r="H110" s="5">
         <v>18</v>
       </c>
-      <c r="I110">
+      <c r="I110" s="5">
         <v>2</v>
       </c>
       <c r="J110">
@@ -6368,10 +6380,10 @@
       <c r="G111">
         <v>0</v>
       </c>
-      <c r="H111">
+      <c r="H111" s="5">
         <v>3.2183908045976999</v>
       </c>
-      <c r="I111">
+      <c r="I111" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J111">
@@ -6407,10 +6419,10 @@
       <c r="G112">
         <v>0</v>
       </c>
-      <c r="H112">
+      <c r="H112" s="5">
         <v>192</v>
       </c>
-      <c r="I112">
+      <c r="I112" s="5">
         <v>2</v>
       </c>
       <c r="J112">
@@ -6446,10 +6458,10 @@
       <c r="G113">
         <v>0</v>
       </c>
-      <c r="H113">
+      <c r="H113" s="5">
         <v>192</v>
       </c>
-      <c r="I113">
+      <c r="I113" s="5">
         <v>2</v>
       </c>
       <c r="J113">
@@ -6485,10 +6497,10 @@
       <c r="G114">
         <v>1</v>
       </c>
-      <c r="H114">
+      <c r="H114" s="5">
         <v>168</v>
       </c>
-      <c r="I114">
+      <c r="I114" s="5">
         <v>2</v>
       </c>
       <c r="J114">
@@ -6524,10 +6536,10 @@
       <c r="G115">
         <v>1</v>
       </c>
-      <c r="H115">
+      <c r="H115" s="5">
         <v>144</v>
       </c>
-      <c r="I115">
+      <c r="I115" s="5">
         <v>2</v>
       </c>
       <c r="J115">
@@ -6557,10 +6569,10 @@
       <c r="G116">
         <v>0</v>
       </c>
-      <c r="H116">
+      <c r="H116" s="5">
         <v>60</v>
       </c>
-      <c r="I116">
+      <c r="I116" s="5">
         <v>2</v>
       </c>
       <c r="J116">
@@ -6590,10 +6602,10 @@
       <c r="G117">
         <v>0</v>
       </c>
-      <c r="H117">
+      <c r="H117" s="5">
         <v>156</v>
       </c>
-      <c r="I117">
+      <c r="I117" s="5">
         <v>2</v>
       </c>
       <c r="J117">
@@ -6623,10 +6635,10 @@
       <c r="G118">
         <v>0</v>
       </c>
-      <c r="H118">
+      <c r="H118" s="5">
         <v>24</v>
       </c>
-      <c r="I118">
+      <c r="I118" s="5">
         <v>2</v>
       </c>
       <c r="J118">
@@ -6656,10 +6668,10 @@
       <c r="G119">
         <v>0</v>
       </c>
-      <c r="H119">
+      <c r="H119" s="5">
         <v>3.2183908045976999</v>
       </c>
-      <c r="I119">
+      <c r="I119" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J119">
@@ -6689,10 +6701,10 @@
       <c r="G120">
         <v>0</v>
       </c>
-      <c r="H120">
+      <c r="H120" s="5">
         <v>48</v>
       </c>
-      <c r="I120">
+      <c r="I120" s="5">
         <v>2</v>
       </c>
       <c r="J120">
@@ -6728,10 +6740,10 @@
       <c r="G121">
         <v>0</v>
       </c>
-      <c r="H121">
+      <c r="H121" s="5">
         <v>48</v>
       </c>
-      <c r="I121">
+      <c r="I121" s="5">
         <v>2</v>
       </c>
       <c r="J121">
@@ -6761,10 +6773,10 @@
       <c r="G122">
         <v>0</v>
       </c>
-      <c r="H122">
+      <c r="H122" s="5">
         <v>144</v>
       </c>
-      <c r="I122">
+      <c r="I122" s="5">
         <v>2</v>
       </c>
       <c r="J122">
@@ -6794,10 +6806,10 @@
       <c r="G123">
         <v>0</v>
       </c>
-      <c r="H123">
+      <c r="H123" s="5">
         <v>84</v>
       </c>
-      <c r="I123">
+      <c r="I123" s="5">
         <v>2</v>
       </c>
       <c r="J123">
@@ -6827,10 +6839,10 @@
       <c r="G124">
         <v>0</v>
       </c>
-      <c r="H124">
+      <c r="H124" s="5">
         <v>3.2183908045976999</v>
       </c>
-      <c r="I124">
+      <c r="I124" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J124">
@@ -6860,10 +6872,10 @@
       <c r="G125">
         <v>0</v>
       </c>
-      <c r="H125">
+      <c r="H125" s="5">
         <v>18</v>
       </c>
-      <c r="I125">
+      <c r="I125" s="5">
         <v>2</v>
       </c>
       <c r="J125">
@@ -6893,10 +6905,10 @@
       <c r="G126">
         <v>0</v>
       </c>
-      <c r="H126">
+      <c r="H126" s="5">
         <v>18</v>
       </c>
-      <c r="I126">
+      <c r="I126" s="5">
         <v>2</v>
       </c>
       <c r="J126">
@@ -6926,10 +6938,10 @@
       <c r="G127">
         <v>0</v>
       </c>
-      <c r="H127">
+      <c r="H127" s="5">
         <v>72</v>
       </c>
-      <c r="I127">
+      <c r="I127" s="5">
         <v>2.0689655172413799</v>
       </c>
       <c r="J127">
@@ -6959,10 +6971,10 @@
       <c r="G128">
         <v>0</v>
       </c>
-      <c r="H128">
-        <v>4</v>
-      </c>
-      <c r="I128">
+      <c r="H128" s="5">
+        <v>4</v>
+      </c>
+      <c r="I128" s="5">
         <v>2</v>
       </c>
       <c r="J128">
@@ -6992,10 +7004,10 @@
       <c r="G129">
         <v>0</v>
       </c>
-      <c r="H129">
+      <c r="H129" s="5">
         <v>216</v>
       </c>
-      <c r="I129">
+      <c r="I129" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J129">
@@ -7025,10 +7037,10 @@
       <c r="G130">
         <v>0</v>
       </c>
-      <c r="H130">
-        <v>4</v>
-      </c>
-      <c r="I130">
+      <c r="H130" s="5">
+        <v>4</v>
+      </c>
+      <c r="I130" s="5">
         <v>2</v>
       </c>
       <c r="J130">
@@ -7058,10 +7070,10 @@
       <c r="G131">
         <v>0</v>
       </c>
-      <c r="H131">
+      <c r="H131" s="5">
         <v>3.2183908045976999</v>
       </c>
-      <c r="I131">
+      <c r="I131" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J131">
@@ -7091,10 +7103,10 @@
       <c r="G132">
         <v>0</v>
       </c>
-      <c r="H132">
+      <c r="H132" s="5">
         <v>18</v>
       </c>
-      <c r="I132">
+      <c r="I132" s="5">
         <v>2</v>
       </c>
       <c r="J132">
@@ -7130,10 +7142,10 @@
       <c r="G133">
         <v>0</v>
       </c>
-      <c r="H133">
+      <c r="H133" s="5">
         <v>132</v>
       </c>
-      <c r="I133">
+      <c r="I133" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J133">
@@ -7163,10 +7175,10 @@
       <c r="G134">
         <v>0</v>
       </c>
-      <c r="H134">
+      <c r="H134" s="5">
         <v>3.2183908045976999</v>
       </c>
-      <c r="I134">
+      <c r="I134" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J134">
@@ -7196,10 +7208,10 @@
       <c r="G135">
         <v>0</v>
       </c>
-      <c r="H135">
+      <c r="H135" s="5">
         <v>18</v>
       </c>
-      <c r="I135">
+      <c r="I135" s="5">
         <v>2</v>
       </c>
       <c r="J135">
@@ -7229,10 +7241,10 @@
       <c r="G136">
         <v>0</v>
       </c>
-      <c r="H136">
+      <c r="H136" s="5">
         <v>3.2183908045976999</v>
       </c>
-      <c r="I136">
+      <c r="I136" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J136">
@@ -7262,10 +7274,10 @@
       <c r="G137">
         <v>0</v>
       </c>
-      <c r="H137">
+      <c r="H137" s="5">
         <v>132</v>
       </c>
-      <c r="I137">
+      <c r="I137" s="5">
         <v>2</v>
       </c>
       <c r="J137">
@@ -7295,10 +7307,10 @@
       <c r="G138">
         <v>0</v>
       </c>
-      <c r="H138">
+      <c r="H138" s="5">
         <v>3.2183908045976999</v>
       </c>
-      <c r="I138">
+      <c r="I138" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J138">
@@ -7328,10 +7340,10 @@
       <c r="G139">
         <v>0</v>
       </c>
-      <c r="H139">
+      <c r="H139" s="5">
         <v>3.2183908045976999</v>
       </c>
-      <c r="I139">
+      <c r="I139" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J139">
@@ -7361,10 +7373,10 @@
       <c r="G140">
         <v>0</v>
       </c>
-      <c r="H140">
+      <c r="H140" s="5">
         <v>72</v>
       </c>
-      <c r="I140">
+      <c r="I140" s="5">
         <v>2</v>
       </c>
       <c r="J140">
@@ -7400,10 +7412,10 @@
       <c r="G141">
         <v>0</v>
       </c>
-      <c r="H141">
+      <c r="H141" s="5">
         <v>132</v>
       </c>
-      <c r="I141">
+      <c r="I141" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J141">
@@ -7439,10 +7451,10 @@
       <c r="G142">
         <v>1</v>
       </c>
-      <c r="H142">
+      <c r="H142" s="5">
         <v>48</v>
       </c>
-      <c r="I142">
+      <c r="I142" s="5">
         <v>3</v>
       </c>
       <c r="J142">
@@ -7478,10 +7490,10 @@
       <c r="G143">
         <v>1</v>
       </c>
-      <c r="H143">
+      <c r="H143" s="5">
         <v>180</v>
       </c>
-      <c r="I143">
+      <c r="I143" s="5">
         <v>3</v>
       </c>
       <c r="J143">
@@ -7511,10 +7523,10 @@
       <c r="G144">
         <v>0</v>
       </c>
-      <c r="H144">
+      <c r="H144" s="5">
         <v>3.2183908045976999</v>
       </c>
-      <c r="I144">
+      <c r="I144" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J144">
@@ -7544,10 +7556,10 @@
       <c r="G145">
         <v>0</v>
       </c>
-      <c r="H145">
+      <c r="H145" s="5">
         <v>48</v>
       </c>
-      <c r="I145">
+      <c r="I145" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J145">
@@ -7583,10 +7595,10 @@
       <c r="G146">
         <v>1</v>
       </c>
-      <c r="H146">
+      <c r="H146" s="5">
         <v>156</v>
       </c>
-      <c r="I146">
+      <c r="I146" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J146">
@@ -7622,10 +7634,10 @@
       <c r="G147">
         <v>1</v>
       </c>
-      <c r="H147">
+      <c r="H147" s="5">
         <v>18</v>
       </c>
-      <c r="I147">
+      <c r="I147" s="5">
         <v>2</v>
       </c>
       <c r="J147">
@@ -7661,10 +7673,10 @@
       <c r="G148">
         <v>0</v>
       </c>
-      <c r="H148">
+      <c r="H148" s="5">
         <v>3.2183908045976999</v>
       </c>
-      <c r="I148">
+      <c r="I148" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J148">
@@ -7700,10 +7712,10 @@
       <c r="G149">
         <v>1</v>
       </c>
-      <c r="H149">
+      <c r="H149" s="5">
         <v>120</v>
       </c>
-      <c r="I149">
+      <c r="I149" s="5">
         <v>2</v>
       </c>
       <c r="J149">
@@ -7739,10 +7751,10 @@
       <c r="G150">
         <v>0</v>
       </c>
-      <c r="H150">
+      <c r="H150" s="5">
         <v>48</v>
       </c>
-      <c r="I150">
+      <c r="I150" s="5">
         <v>2</v>
       </c>
       <c r="J150">
@@ -7778,10 +7790,10 @@
       <c r="G151">
         <v>0</v>
       </c>
-      <c r="H151">
+      <c r="H151" s="5">
         <v>3.2183908045976999</v>
       </c>
-      <c r="I151">
+      <c r="I151" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J151">
@@ -7811,10 +7823,10 @@
       <c r="G152">
         <v>0</v>
       </c>
-      <c r="H152">
+      <c r="H152" s="5">
         <v>120</v>
       </c>
-      <c r="I152">
+      <c r="I152" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J152">
@@ -7844,10 +7856,10 @@
       <c r="G153">
         <v>0</v>
       </c>
-      <c r="H153">
-        <v>3</v>
-      </c>
-      <c r="I153">
+      <c r="H153" s="5">
+        <v>3</v>
+      </c>
+      <c r="I153" s="5">
         <v>1</v>
       </c>
       <c r="J153">
@@ -7883,10 +7895,10 @@
       <c r="G154">
         <v>1</v>
       </c>
-      <c r="H154">
+      <c r="H154" s="5">
         <v>168</v>
       </c>
-      <c r="I154">
+      <c r="I154" s="5">
         <v>1.6091954022988499</v>
       </c>
       <c r="J154">
@@ -7916,10 +7928,10 @@
       <c r="G155">
         <v>0</v>
       </c>
-      <c r="H155">
+      <c r="H155" s="5">
         <v>3.2183908045976999</v>
       </c>
-      <c r="I155">
+      <c r="I155" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J155">
@@ -7955,10 +7967,10 @@
       <c r="G156">
         <v>0</v>
       </c>
-      <c r="H156">
+      <c r="H156" s="5">
         <v>60</v>
       </c>
-      <c r="I156">
+      <c r="I156" s="5">
         <v>2</v>
       </c>
       <c r="J156">
@@ -7994,10 +8006,10 @@
       <c r="G157">
         <v>1</v>
       </c>
-      <c r="H157">
+      <c r="H157" s="5">
         <v>120</v>
       </c>
-      <c r="I157">
+      <c r="I157" s="5">
         <v>2</v>
       </c>
       <c r="J157">
@@ -8027,10 +8039,10 @@
       <c r="G158">
         <v>0</v>
       </c>
-      <c r="H158">
+      <c r="H158" s="5">
         <v>18</v>
       </c>
-      <c r="I158">
+      <c r="I158" s="5">
         <v>2</v>
       </c>
       <c r="J158">
@@ -8060,10 +8072,10 @@
       <c r="G159">
         <v>0</v>
       </c>
-      <c r="H159">
+      <c r="H159" s="5">
         <v>132</v>
       </c>
-      <c r="I159">
+      <c r="I159" s="5">
         <v>2</v>
       </c>
       <c r="J159">
@@ -8099,10 +8111,10 @@
       <c r="G160">
         <v>0</v>
       </c>
-      <c r="H160">
+      <c r="H160" s="5">
         <v>216</v>
       </c>
-      <c r="I160">
+      <c r="I160" s="5">
         <v>2</v>
       </c>
       <c r="J160">
@@ -8138,10 +8150,10 @@
       <c r="G161">
         <v>0</v>
       </c>
-      <c r="H161">
+      <c r="H161" s="5">
         <v>168</v>
       </c>
-      <c r="I161">
+      <c r="I161" s="5">
         <v>2</v>
       </c>
       <c r="J161">
@@ -8171,10 +8183,10 @@
       <c r="G162">
         <v>1</v>
       </c>
-      <c r="H162">
+      <c r="H162" s="5">
         <v>18</v>
       </c>
-      <c r="I162">
+      <c r="I162" s="5">
         <v>3</v>
       </c>
       <c r="J162">
@@ -8204,10 +8216,10 @@
       <c r="G163">
         <v>0</v>
       </c>
-      <c r="H163">
+      <c r="H163" s="5">
         <v>3.2183908045976999</v>
       </c>
-      <c r="I163">
+      <c r="I163" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J163">
@@ -8243,10 +8255,10 @@
       <c r="G164">
         <v>0</v>
       </c>
-      <c r="H164">
+      <c r="H164" s="5">
         <v>72</v>
       </c>
-      <c r="I164">
+      <c r="I164" s="5">
         <v>2</v>
       </c>
       <c r="J164">
@@ -8276,10 +8288,10 @@
       <c r="G165">
         <v>0</v>
       </c>
-      <c r="H165">
+      <c r="H165" s="5">
         <v>3.2183908045976999</v>
       </c>
-      <c r="I165">
+      <c r="I165" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J165">
@@ -8309,10 +8321,10 @@
       <c r="G166">
         <v>0</v>
       </c>
-      <c r="H166">
+      <c r="H166" s="5">
         <v>3.2183908045976999</v>
       </c>
-      <c r="I166">
+      <c r="I166" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J166">
@@ -8348,10 +8360,10 @@
       <c r="G167">
         <v>0</v>
       </c>
-      <c r="H167">
+      <c r="H167" s="5">
         <v>132</v>
       </c>
-      <c r="I167">
+      <c r="I167" s="5">
         <v>2</v>
       </c>
       <c r="J167">
@@ -8381,10 +8393,10 @@
       <c r="G168">
         <v>0</v>
       </c>
-      <c r="H168">
+      <c r="H168" s="5">
         <v>3.2183908045976999</v>
       </c>
-      <c r="I168">
+      <c r="I168" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J168">
@@ -8414,10 +8426,10 @@
       <c r="G169">
         <v>0</v>
       </c>
-      <c r="H169">
+      <c r="H169" s="5">
         <v>3.2183908045976999</v>
       </c>
-      <c r="I169">
+      <c r="I169" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J169">
@@ -8453,10 +8465,10 @@
       <c r="G170">
         <v>1</v>
       </c>
-      <c r="H170">
+      <c r="H170" s="5">
         <v>48</v>
       </c>
-      <c r="I170">
+      <c r="I170" s="5">
         <v>2</v>
       </c>
       <c r="J170">
@@ -8486,10 +8498,10 @@
       <c r="G171">
         <v>0</v>
       </c>
-      <c r="H171">
+      <c r="H171" s="5">
         <v>180</v>
       </c>
-      <c r="I171">
+      <c r="I171" s="5">
         <v>3</v>
       </c>
       <c r="J171">
@@ -8519,10 +8531,10 @@
       <c r="G172">
         <v>0</v>
       </c>
-      <c r="H172">
+      <c r="H172" s="5">
         <v>3.2183908045976999</v>
       </c>
-      <c r="I172">
+      <c r="I172" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J172">
@@ -8552,10 +8564,10 @@
       <c r="G173">
         <v>0</v>
       </c>
-      <c r="H173">
+      <c r="H173" s="5">
         <v>84</v>
       </c>
-      <c r="I173">
+      <c r="I173" s="5">
         <v>1.83908045977012</v>
       </c>
       <c r="J173">
@@ -8585,10 +8597,10 @@
       <c r="G174">
         <v>0</v>
       </c>
-      <c r="H174">
+      <c r="H174" s="5">
         <v>3.2183908045976999</v>
       </c>
-      <c r="I174">
+      <c r="I174" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J174">
@@ -8618,10 +8630,10 @@
       <c r="G175">
         <v>0</v>
       </c>
-      <c r="H175">
+      <c r="H175" s="5">
         <v>3.2183908045976999</v>
       </c>
-      <c r="I175">
+      <c r="I175" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J175">
@@ -8651,10 +8663,10 @@
       <c r="G176">
         <v>1</v>
       </c>
-      <c r="H176">
+      <c r="H176" s="5">
         <v>60</v>
       </c>
-      <c r="I176">
+      <c r="I176" s="5">
         <v>2</v>
       </c>
       <c r="J176">
@@ -8684,10 +8696,10 @@
       <c r="G177">
         <v>0</v>
       </c>
-      <c r="H177">
+      <c r="H177" s="5">
         <v>144</v>
       </c>
-      <c r="I177">
+      <c r="I177" s="5">
         <v>2</v>
       </c>
       <c r="J177">
@@ -8723,10 +8735,10 @@
       <c r="G178">
         <v>0</v>
       </c>
-      <c r="H178">
+      <c r="H178" s="5">
         <v>96</v>
       </c>
-      <c r="I178">
+      <c r="I178" s="5">
         <v>3</v>
       </c>
       <c r="J178">
@@ -8762,10 +8774,10 @@
       <c r="G179">
         <v>0</v>
       </c>
-      <c r="H179">
+      <c r="H179" s="5">
         <v>192</v>
       </c>
-      <c r="I179">
+      <c r="I179" s="5">
         <v>3</v>
       </c>
       <c r="J179">
@@ -8795,10 +8807,10 @@
       <c r="G180">
         <v>0</v>
       </c>
-      <c r="H180">
+      <c r="H180" s="5">
         <v>18</v>
       </c>
-      <c r="I180">
+      <c r="I180" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J180">
@@ -8828,10 +8840,10 @@
       <c r="G181">
         <v>0</v>
       </c>
-      <c r="H181">
+      <c r="H181" s="5">
         <v>12</v>
       </c>
-      <c r="I181">
+      <c r="I181" s="5">
         <v>2</v>
       </c>
       <c r="J181">
@@ -8861,10 +8873,10 @@
       <c r="G182">
         <v>0</v>
       </c>
-      <c r="H182">
+      <c r="H182" s="5">
         <v>18</v>
       </c>
-      <c r="I182">
+      <c r="I182" s="5">
         <v>3</v>
       </c>
       <c r="J182">
@@ -8894,10 +8906,10 @@
       <c r="G183">
         <v>0</v>
       </c>
-      <c r="H183">
+      <c r="H183" s="5">
         <v>18</v>
       </c>
-      <c r="I183">
+      <c r="I183" s="5">
         <v>1.83908045977012</v>
       </c>
       <c r="J183">
@@ -8927,10 +8939,10 @@
       <c r="G184">
         <v>0</v>
       </c>
-      <c r="H184">
+      <c r="H184" s="5">
         <v>36</v>
       </c>
-      <c r="I184">
+      <c r="I184" s="5">
         <v>2</v>
       </c>
       <c r="J184">
@@ -8960,10 +8972,10 @@
       <c r="G185">
         <v>0</v>
       </c>
-      <c r="H185">
+      <c r="H185" s="5">
         <v>3.2183908045976999</v>
       </c>
-      <c r="I185">
+      <c r="I185" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J185">
@@ -8993,10 +9005,10 @@
       <c r="G186">
         <v>0</v>
       </c>
-      <c r="H186">
+      <c r="H186" s="5">
         <v>3.2183908045976999</v>
       </c>
-      <c r="I186">
+      <c r="I186" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J186">
@@ -9032,10 +9044,10 @@
       <c r="G187">
         <v>0</v>
       </c>
-      <c r="H187">
+      <c r="H187" s="5">
         <v>48</v>
       </c>
-      <c r="I187">
+      <c r="I187" s="5">
         <v>2</v>
       </c>
       <c r="J187">
@@ -9065,10 +9077,10 @@
       <c r="G188">
         <v>0</v>
       </c>
-      <c r="H188">
+      <c r="H188" s="5">
         <v>23</v>
       </c>
-      <c r="I188">
+      <c r="I188" s="5">
         <v>2</v>
       </c>
       <c r="J188">
@@ -9098,10 +9110,10 @@
       <c r="G189">
         <v>0</v>
       </c>
-      <c r="H189">
+      <c r="H189" s="5">
         <v>60</v>
       </c>
-      <c r="I189">
+      <c r="I189" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J189">
@@ -9131,10 +9143,10 @@
       <c r="G190">
         <v>0</v>
       </c>
-      <c r="H190">
+      <c r="H190" s="5">
         <v>18</v>
       </c>
-      <c r="I190">
+      <c r="I190" s="5">
         <v>2</v>
       </c>
       <c r="J190">
@@ -9164,10 +9176,10 @@
       <c r="G191">
         <v>0</v>
       </c>
-      <c r="H191">
+      <c r="H191" s="5">
         <v>18</v>
       </c>
-      <c r="I191">
+      <c r="I191" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J191">
@@ -9197,10 +9209,10 @@
       <c r="G192">
         <v>0</v>
       </c>
-      <c r="H192">
+      <c r="H192" s="5">
         <v>60</v>
       </c>
-      <c r="I192">
+      <c r="I192" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J192">
@@ -9230,10 +9242,10 @@
       <c r="G193">
         <v>0</v>
       </c>
-      <c r="H193">
+      <c r="H193" s="5">
         <v>60</v>
       </c>
-      <c r="I193">
+      <c r="I193" s="5">
         <v>2</v>
       </c>
       <c r="J193">
@@ -9263,10 +9275,10 @@
       <c r="G194">
         <v>0</v>
       </c>
-      <c r="H194">
+      <c r="H194" s="5">
         <v>18</v>
       </c>
-      <c r="I194">
+      <c r="I194" s="5">
         <v>2</v>
       </c>
       <c r="J194">
@@ -9296,10 +9308,10 @@
       <c r="G195">
         <v>0</v>
       </c>
-      <c r="H195">
+      <c r="H195" s="5">
         <v>48</v>
       </c>
-      <c r="I195">
+      <c r="I195" s="5">
         <v>2</v>
       </c>
       <c r="J195">
@@ -9329,10 +9341,10 @@
       <c r="G196">
         <v>0</v>
       </c>
-      <c r="H196">
+      <c r="H196" s="5">
         <v>72</v>
       </c>
-      <c r="I196">
+      <c r="I196" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J196">
@@ -9362,10 +9374,10 @@
       <c r="G197">
         <v>0</v>
       </c>
-      <c r="H197">
+      <c r="H197" s="5">
         <v>3.2183908045976999</v>
       </c>
-      <c r="I197">
+      <c r="I197" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J197">
@@ -9395,10 +9407,10 @@
       <c r="G198">
         <v>0</v>
       </c>
-      <c r="H198">
+      <c r="H198" s="5">
         <v>3.2183908045976999</v>
       </c>
-      <c r="I198">
+      <c r="I198" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J198">
@@ -9428,10 +9440,10 @@
       <c r="G199">
         <v>0</v>
       </c>
-      <c r="H199">
+      <c r="H199" s="5">
         <v>18</v>
       </c>
-      <c r="I199">
+      <c r="I199" s="5">
         <v>2</v>
       </c>
       <c r="J199">
@@ -9467,10 +9479,10 @@
       <c r="G200">
         <v>1</v>
       </c>
-      <c r="H200">
+      <c r="H200" s="5">
         <v>132</v>
       </c>
-      <c r="I200">
+      <c r="I200" s="5">
         <v>2</v>
       </c>
       <c r="J200">
@@ -9506,10 +9518,10 @@
       <c r="G201">
         <v>0</v>
       </c>
-      <c r="H201">
+      <c r="H201" s="5">
         <v>144</v>
       </c>
-      <c r="I201">
+      <c r="I201" s="5">
         <v>2</v>
       </c>
       <c r="J201">
@@ -9539,10 +9551,10 @@
       <c r="G202">
         <v>0</v>
       </c>
-      <c r="H202">
+      <c r="H202" s="5">
         <v>16</v>
       </c>
-      <c r="I202">
+      <c r="I202" s="5">
         <v>2</v>
       </c>
       <c r="J202">
@@ -9572,10 +9584,10 @@
       <c r="G203">
         <v>0</v>
       </c>
-      <c r="H203">
+      <c r="H203" s="5">
         <v>18</v>
       </c>
-      <c r="I203">
+      <c r="I203" s="5">
         <v>2</v>
       </c>
       <c r="J203">
@@ -9605,10 +9617,10 @@
       <c r="G204">
         <v>0</v>
       </c>
-      <c r="H204">
+      <c r="H204" s="5">
         <v>60</v>
       </c>
-      <c r="I204">
+      <c r="I204" s="5">
         <v>2</v>
       </c>
       <c r="J204">
@@ -9644,10 +9656,10 @@
       <c r="G205">
         <v>0</v>
       </c>
-      <c r="H205">
+      <c r="H205" s="5">
         <v>48</v>
       </c>
-      <c r="I205">
+      <c r="I205" s="5">
         <v>2</v>
       </c>
       <c r="J205">
@@ -9677,10 +9689,10 @@
       <c r="G206">
         <v>0</v>
       </c>
-      <c r="H206">
+      <c r="H206" s="5">
         <v>18</v>
       </c>
-      <c r="I206">
+      <c r="I206" s="5">
         <v>2</v>
       </c>
       <c r="J206">
@@ -9710,10 +9722,10 @@
       <c r="G207">
         <v>0</v>
       </c>
-      <c r="H207">
+      <c r="H207" s="5">
         <v>3.2183908045976999</v>
       </c>
-      <c r="I207">
+      <c r="I207" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J207">
@@ -9743,10 +9755,10 @@
       <c r="G208">
         <v>0</v>
       </c>
-      <c r="H208">
+      <c r="H208" s="5">
         <v>72</v>
       </c>
-      <c r="I208">
+      <c r="I208" s="5">
         <v>2</v>
       </c>
       <c r="J208">
@@ -9776,10 +9788,10 @@
       <c r="G209">
         <v>0</v>
       </c>
-      <c r="H209">
+      <c r="H209" s="5">
         <v>15</v>
       </c>
-      <c r="I209">
+      <c r="I209" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J209">
@@ -9809,10 +9821,10 @@
       <c r="G210">
         <v>0</v>
       </c>
-      <c r="H210">
+      <c r="H210" s="5">
         <v>12</v>
       </c>
-      <c r="I210">
+      <c r="I210" s="5">
         <v>2</v>
       </c>
       <c r="J210">
@@ -9842,10 +9854,10 @@
       <c r="G211">
         <v>0</v>
       </c>
-      <c r="H211">
+      <c r="H211" s="5">
         <v>84</v>
       </c>
-      <c r="I211">
+      <c r="I211" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J211">
@@ -9881,10 +9893,10 @@
       <c r="G212">
         <v>0</v>
       </c>
-      <c r="H212">
+      <c r="H212" s="5">
         <v>18</v>
       </c>
-      <c r="I212">
+      <c r="I212" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J212">
@@ -9914,10 +9926,10 @@
       <c r="G213">
         <v>0</v>
       </c>
-      <c r="H213">
+      <c r="H213" s="5">
         <v>3.2183908045976999</v>
       </c>
-      <c r="I213">
+      <c r="I213" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J213">
@@ -9947,10 +9959,10 @@
       <c r="G214">
         <v>0</v>
       </c>
-      <c r="H214">
+      <c r="H214" s="5">
         <v>18</v>
       </c>
-      <c r="I214">
+      <c r="I214" s="5">
         <v>1.3793103448275901</v>
       </c>
       <c r="J214">

</xml_diff>